<commit_message>
Update berita 2026-08-03 12:48 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-29.xlsx
+++ b/data/berita_antara_2026-07-29.xlsx
@@ -471,66 +471,66 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>hukum</t>
+          <t>ekonomi-bursa</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Daftar 7 Kejaksaan Negeri baru yang dibentuk Prabowo, ini lokasi dan tujuannya</t>
+          <t>IHSG ditutup melemah terbebani sentimen global dan domestik</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 07:22:43 +0700</t>
+          <t>Wed, 29 Jul 2026 16:47:51 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto membentuk tujuh Kejaksaan Negeri (Kejari) baru melalui Peraturan Presiden (Perpres) Nomor 40 ...</t>
+          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Rabu sore ditutup melemah terbebani oleh sentimen ...</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5670295/daftar-7-kejaksaan-negeri-baru-yang-dibentuk-prabowo-ini-lokasi-dan-tujuannya</t>
+          <t>https://www.antaranews.com/berita/5671131/ihsg-ditutup-melemah-terbebani-sentimen-global-dan-domestik</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/24/1000086234.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-02.jpg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ekonomi-bursa</t>
+          <t>hukum</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>OJK: Penghimpunan dana di pasar modal tetap positif hingga akhir 2026</t>
+          <t>Daftar 7 Kejaksaan Negeri baru yang dibentuk Prabowo, ini lokasi dan tujuannya</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 23:02:38 +0700</t>
+          <t>Wed, 29 Jul 2026 07:22:43 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) memandang prospek penghimpunan dana di pasar modal hingga akhir tahun 2026 tetap positif ...</t>
+          <t>Presiden Prabowo Subianto membentuk tujuh Kejaksaan Negeri (Kejari) baru melalui Peraturan Presiden (Perpres) Nomor 40 ...</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5671813/ojk-penghimpunan-dana-di-pasar-modal-tetap-positif-hingga-akhir-2026</t>
+          <t>https://www.antaranews.com/berita/5670295/daftar-7-kejaksaan-negeri-baru-yang-dibentuk-prabowo-ini-lokasi-dan-tujuannya</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/24/1000086234.jpg</t>
         </is>
       </c>
     </row>
@@ -542,28 +542,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>OJK: Aliran dana asing dipengaruhi geopolitik dan suku bunga global</t>
+          <t>OJK: Penghimpunan dana di pasar modal tetap positif hingga akhir 2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 21:19:21 +0700</t>
+          <t>Wed, 29 Jul 2026 23:02:38 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Kepala Eksekutif Pengawas Pasar Modal, Keuangan Derivatif dan Bursa Karbon (PMDK) Otoritas Jasa Keuangan (OJK) Hasan ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) memandang prospek penghimpunan dana di pasar modal hingga akhir tahun 2026 tetap positif ...</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5671679/ojk-aliran-dana-asing-dipengaruhi-geopolitik-dan-suku-bunga-global</t>
+          <t>https://www.antaranews.com/berita/5671813/ojk-penghimpunan-dana-di-pasar-modal-tetap-positif-hingga-akhir-2026</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/03/WhatsApp-Image-2026-07-03-at-11.17.02.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
         </is>
       </c>
     </row>
@@ -575,28 +575,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OJK targetkan POJK demutualisasi BEI tuntas pekan kedua September 2026</t>
+          <t>OJK: Aliran dana asing dipengaruhi geopolitik dan suku bunga global</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 18:44:11 +0700</t>
+          <t>Wed, 29 Jul 2026 21:19:21 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) menargetkan Peraturan OJK (POJK) turunan Undang-Undang Nomor 4 Tahun 2026 (Revisi UU P2SK) ...</t>
+          <t>Kepala Eksekutif Pengawas Pasar Modal, Keuangan Derivatif dan Bursa Karbon (PMDK) Otoritas Jasa Keuangan (OJK) Hasan ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5671364/ojk-targetkan-pojk-demutualisasi-bei-tuntas-pekan-kedua-september-2026</t>
+          <t>https://www.antaranews.com/berita/5671679/ojk-aliran-dana-asing-dipengaruhi-geopolitik-dan-suku-bunga-global</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-16.42.53.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/03/WhatsApp-Image-2026-07-03-at-11.17.02.jpeg</t>
         </is>
       </c>
     </row>
@@ -608,28 +608,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>IHSG ditutup melemah terbebani sentimen global dan domestik</t>
+          <t>OJK targetkan POJK demutualisasi BEI tuntas pekan kedua September 2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 16:47:51 +0700</t>
+          <t>Wed, 29 Jul 2026 18:44:11 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Rabu sore ditutup melemah terbebani oleh sentimen ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) menargetkan Peraturan OJK (POJK) turunan Undang-Undang Nomor 4 Tahun 2026 (Revisi UU P2SK) ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5671131/ihsg-ditutup-melemah-terbebani-sentimen-global-dan-domestik</t>
+          <t>https://www.antaranews.com/berita/5671364/ojk-targetkan-pojk-demutualisasi-bei-tuntas-pekan-kedua-september-2026</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-02.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-16.42.53.jpeg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update berita 2026-08-03 15:35 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-29.xlsx
+++ b/data/berita_antara_2026-07-29.xlsx
@@ -504,33 +504,33 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hukum</t>
+          <t>ekonomi-bursa</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Daftar 7 Kejaksaan Negeri baru yang dibentuk Prabowo, ini lokasi dan tujuannya</t>
+          <t>OJK: Aliran dana asing dipengaruhi geopolitik dan suku bunga global</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 07:22:43 +0700</t>
+          <t>Wed, 29 Jul 2026 21:19:21 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto membentuk tujuh Kejaksaan Negeri (Kejari) baru melalui Peraturan Presiden (Perpres) Nomor 40 ...</t>
+          <t>Kepala Eksekutif Pengawas Pasar Modal, Keuangan Derivatif dan Bursa Karbon (PMDK) Otoritas Jasa Keuangan (OJK) Hasan ...</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5670295/daftar-7-kejaksaan-negeri-baru-yang-dibentuk-prabowo-ini-lokasi-dan-tujuannya</t>
+          <t>https://www.antaranews.com/berita/5671679/ojk-aliran-dana-asing-dipengaruhi-geopolitik-dan-suku-bunga-global</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/24/1000086234.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/03/WhatsApp-Image-2026-07-03-at-11.17.02.jpeg</t>
         </is>
       </c>
     </row>
@@ -542,61 +542,61 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>OJK: Penghimpunan dana di pasar modal tetap positif hingga akhir 2026</t>
+          <t>OJK targetkan POJK demutualisasi BEI tuntas pekan kedua September 2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 23:02:38 +0700</t>
+          <t>Wed, 29 Jul 2026 18:44:11 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) memandang prospek penghimpunan dana di pasar modal hingga akhir tahun 2026 tetap positif ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) menargetkan Peraturan OJK (POJK) turunan Undang-Undang Nomor 4 Tahun 2026 (Revisi UU P2SK) ...</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5671813/ojk-penghimpunan-dana-di-pasar-modal-tetap-positif-hingga-akhir-2026</t>
+          <t>https://www.antaranews.com/berita/5671364/ojk-targetkan-pojk-demutualisasi-bei-tuntas-pekan-kedua-september-2026</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-16.42.53.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ekonomi-bursa</t>
+          <t>hukum</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OJK: Aliran dana asing dipengaruhi geopolitik dan suku bunga global</t>
+          <t>Daftar 7 Kejaksaan Negeri baru yang dibentuk Prabowo, ini lokasi dan tujuannya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 21:19:21 +0700</t>
+          <t>Wed, 29 Jul 2026 07:22:43 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Kepala Eksekutif Pengawas Pasar Modal, Keuangan Derivatif dan Bursa Karbon (PMDK) Otoritas Jasa Keuangan (OJK) Hasan ...</t>
+          <t>Presiden Prabowo Subianto membentuk tujuh Kejaksaan Negeri (Kejari) baru melalui Peraturan Presiden (Perpres) Nomor 40 ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5671679/ojk-aliran-dana-asing-dipengaruhi-geopolitik-dan-suku-bunga-global</t>
+          <t>https://www.antaranews.com/berita/5670295/daftar-7-kejaksaan-negeri-baru-yang-dibentuk-prabowo-ini-lokasi-dan-tujuannya</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/03/WhatsApp-Image-2026-07-03-at-11.17.02.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/24/1000086234.jpg</t>
         </is>
       </c>
     </row>
@@ -608,28 +608,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>OJK targetkan POJK demutualisasi BEI tuntas pekan kedua September 2026</t>
+          <t>OJK: Penghimpunan dana di pasar modal tetap positif hingga akhir 2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 18:44:11 +0700</t>
+          <t>Wed, 29 Jul 2026 23:02:38 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) menargetkan Peraturan OJK (POJK) turunan Undang-Undang Nomor 4 Tahun 2026 (Revisi UU P2SK) ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) memandang prospek penghimpunan dana di pasar modal hingga akhir tahun 2026 tetap positif ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5671364/ojk-targetkan-pojk-demutualisasi-bei-tuntas-pekan-kedua-september-2026</t>
+          <t>https://www.antaranews.com/berita/5671813/ojk-penghimpunan-dana-di-pasar-modal-tetap-positif-hingga-akhir-2026</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-16.42.53.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update berita 2026-08-04 04:52 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-29.xlsx
+++ b/data/berita_antara_2026-07-29.xlsx
@@ -570,66 +570,66 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>hukum</t>
+          <t>ekonomi-bursa</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Daftar 7 Kejaksaan Negeri baru yang dibentuk Prabowo, ini lokasi dan tujuannya</t>
+          <t>OJK: Penghimpunan dana di pasar modal tetap positif hingga akhir 2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 07:22:43 +0700</t>
+          <t>Wed, 29 Jul 2026 23:02:38 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto membentuk tujuh Kejaksaan Negeri (Kejari) baru melalui Peraturan Presiden (Perpres) Nomor 40 ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) memandang prospek penghimpunan dana di pasar modal hingga akhir tahun 2026 tetap positif ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5670295/daftar-7-kejaksaan-negeri-baru-yang-dibentuk-prabowo-ini-lokasi-dan-tujuannya</t>
+          <t>https://www.antaranews.com/berita/5671813/ojk-penghimpunan-dana-di-pasar-modal-tetap-positif-hingga-akhir-2026</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/24/1000086234.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ekonomi-bursa</t>
+          <t>hukum</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>OJK: Penghimpunan dana di pasar modal tetap positif hingga akhir 2026</t>
+          <t>Daftar 7 Kejaksaan Negeri baru yang dibentuk Prabowo, ini lokasi dan tujuannya</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 23:02:38 +0700</t>
+          <t>Wed, 29 Jul 2026 07:22:43 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) memandang prospek penghimpunan dana di pasar modal hingga akhir tahun 2026 tetap positif ...</t>
+          <t>Presiden Prabowo Subianto membentuk tujuh Kejaksaan Negeri (Kejari) baru melalui Peraturan Presiden (Perpres) Nomor 40 ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5671813/ojk-penghimpunan-dana-di-pasar-modal-tetap-positif-hingga-akhir-2026</t>
+          <t>https://www.antaranews.com/berita/5670295/daftar-7-kejaksaan-negeri-baru-yang-dibentuk-prabowo-ini-lokasi-dan-tujuannya</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/24/1000086234.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update berita 2026-08-04 07:10 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-29.xlsx
+++ b/data/berita_antara_2026-07-29.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Berita" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -429,6 +429,7 @@
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -467,6 +468,11 @@
           <t>URL Gambar</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -500,6 +506,7 @@
           <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-02.jpg</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -533,6 +540,7 @@
           <t>https://cdn.antaranews.com/cache/800x533/2026/07/03/WhatsApp-Image-2026-07-03-at-11.17.02.jpeg</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -566,6 +574,7 @@
           <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-16.42.53.jpeg</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -599,6 +608,7 @@
           <t>https://cdn.antaranews.com/cache/800x533/2026/06/30/WhatsApp-Image-2026-06-30-at-18.00.00.jpeg</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -632,6 +642,11 @@
           <t>https://cdn.antaranews.com/cache/800x533/2026/07/24/1000086234.jpg</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -665,6 +680,11 @@
           <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/WhatsApp-Image-2026-07-29-at-20.16.31_1.jpeg</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -698,6 +718,11 @@
           <t>https://cdn.antaranews.com/cache/800x533/2021/12/22/2021-12-21T164847Z_1_LYNXMPEHBK0RK_RTROPTP_4_SOCCER-JAPAN-KING-KAZU.jpg</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -731,6 +756,11 @@
           <t>https://cdn.antaranews.com/cache/800x533/2026/07/28/timnas-indonesia-kalahkan-kamboja-2829197.jpg</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -764,6 +794,11 @@
           <t>https://cdn.antaranews.com/cache/800x533/2026/07/28/Piala-AFF-Indonesia-Lawan-Kamboja-270726-bay-7.jpg</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -797,6 +832,11 @@
           <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/IMG_8481.jpg</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -830,6 +870,11 @@
           <t>https://cdn.antaranews.com/cache/800x533/2026/07/13/IMG-20260713-WA0009.jpg</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -863,6 +908,11 @@
           <t>https://cdn.antaranews.com/cache/800x533/2026/03/20/1000292384.jpg</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -896,6 +946,11 @@
           <t>https://cdn.antaranews.com/cache/800x533/2024/04/26/1000102769.jpg</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -929,6 +984,11 @@
           <t>https://cdn.antaranews.com/cache/800x533/2024/01/07/IMG-20240107-WA0013.jpg</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -962,9 +1022,14 @@
           <t>https://cdn.antaranews.com/cache/800x533/2026/06/29/InShot_20260629_204048450.jpg</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>antara</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G16"/>
+  <autoFilter ref="A1:H16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-05 01:19 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-29.xlsx
+++ b/data/berita_antara_2026-07-29.xlsx
@@ -651,33 +651,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>metro</t>
+          <t>sepakbola</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Polisi buru bandar sabu pemasok dua pengedar di Jakarta Utara</t>
+          <t>Kazuyoshi Miura cetak gol di usia 59 tahun, berikut kisah Sang "King Kazu"</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 20:47:46 +0700</t>
+          <t>Wed, 29 Jul 2026 08:13:28 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Polsek Kawasan Sunda Kelapa, Jakarta Utara, masih memburu seorang bandar narkotika jenis sabu berinisial PN yang ...</t>
+          <t>Usia hanyalah angka bagi Kazuyoshi Miura. Di usianya yang ke 59, ia masih membuktikan kemampuannya setelah mencetak gol ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5671636/polisi-buru-bandar-sabu-pemasok-dua-pengedar-di-jakarta-utara</t>
+          <t>https://www.antaranews.com/berita/5670327/kazuyoshi-miura-cetak-gol-di-usia-59-tahun-berikut-kisah-sang-king-kazu</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/WhatsApp-Image-2026-07-29-at-20.16.31_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2021/12/22/2021-12-21T164847Z_1_LYNXMPEHBK0RK_RTROPTP_4_SOCCER-JAPAN-KING-KAZU.jpg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -694,28 +694,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kazuyoshi Miura cetak gol di usia 59 tahun, berikut kisah Sang "King Kazu"</t>
+          <t>Jadwal Timnas Indonesia vs Timor Leste di Piala AFF 2026, tayang jam berapa dan di mana?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 08:13:28 +0700</t>
+          <t>Wed, 29 Jul 2026 07:34:02 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Usia hanyalah angka bagi Kazuyoshi Miura. Di usianya yang ke 59, ia masih membuktikan kemampuannya setelah mencetak gol ...</t>
+          <t>Timnas Indonesia akan melanjutkan perjuangannya di Grup A Piala AFF 2026 dengan menghadapi Timor Leste pada ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5670327/kazuyoshi-miura-cetak-gol-di-usia-59-tahun-berikut-kisah-sang-king-kazu</t>
+          <t>https://www.antaranews.com/berita/5670304/jadwal-timnas-indonesia-vs-timor-leste-di-piala-aff-2026-tayang-jam-berapa-dan-di-mana</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2021/12/22/2021-12-21T164847Z_1_LYNXMPEHBK0RK_RTROPTP_4_SOCCER-JAPAN-KING-KAZU.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/28/timnas-indonesia-kalahkan-kamboja-2829197.jpg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -732,28 +732,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Jadwal Timnas Indonesia vs Timor Leste di Piala AFF 2026, tayang jam berapa dan di mana?</t>
+          <t>Profil Mitchell Lee Baker, striker naturalisasi Timnas Indonesia yang cetak hattrick di debut</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 07:34:02 +0700</t>
+          <t>Wed, 29 Jul 2026 07:28:58 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Timnas Indonesia akan melanjutkan perjuangannya di Grup A Piala AFF 2026 dengan menghadapi Timor Leste pada ...</t>
+          <t>Mitchell Lee Baker tak butuh waktu lama untuk mencuri perhatian publik sepak bola Indonesia. Penyerang muda berusia 19 ...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5670304/jadwal-timnas-indonesia-vs-timor-leste-di-piala-aff-2026-tayang-jam-berapa-dan-di-mana</t>
+          <t>https://www.antaranews.com/berita/5670297/profil-mitchell-lee-baker-striker-naturalisasi-timnas-indonesia-yang-cetak-hattrick-di-debut</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/28/timnas-indonesia-kalahkan-kamboja-2829197.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/28/Piala-AFF-Indonesia-Lawan-Kamboja-270726-bay-7.jpg</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -765,33 +765,33 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>sepakbola</t>
+          <t>humaniora</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Profil Mitchell Lee Baker, striker naturalisasi Timnas Indonesia yang cetak hattrick di debut</t>
+          <t>Cara ubah desil DTSEN di aplikasi Cek Bansos 2026, simak syarat dan langkah-langkahnya</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 07:28:58 +0700</t>
+          <t>Wed, 29 Jul 2026 07:15:33 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Mitchell Lee Baker tak butuh waktu lama untuk mencuri perhatian publik sepak bola Indonesia. Penyerang muda berusia 19 ...</t>
+          <t>Masyarakat yang merasa data tingkat kesejahteraannya tidak sesuai dalam Data Tunggal Sosial Ekonomi Nasional (DTSEN) ...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5670297/profil-mitchell-lee-baker-striker-naturalisasi-timnas-indonesia-yang-cetak-hattrick-di-debut</t>
+          <t>https://www.antaranews.com/berita/5670292/cara-ubah-desil-dtsen-di-aplikasi-cek-bansos-2026-simak-syarat-dan-langkah-langkahnya</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/28/Piala-AFF-Indonesia-Lawan-Kamboja-270726-bay-7.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/IMG_8481.jpg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -808,28 +808,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cara ubah desil DTSEN di aplikasi Cek Bansos 2026, simak syarat dan langkah-langkahnya</t>
+          <t>Daftar bansos yang masih cair tahun ini, lengkap dengan syaratnya</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 07:15:33 +0700</t>
+          <t>Wed, 29 Jul 2026 07:11:38 +0700</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Masyarakat yang merasa data tingkat kesejahteraannya tidak sesuai dalam Data Tunggal Sosial Ekonomi Nasional (DTSEN) ...</t>
+          <t>Pemerintah masih melanjutkan penyaluran sejumlah program bantuan sosial (bansos) sepanjang 2026 untuk membantu ...</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5670292/cara-ubah-desil-dtsen-di-aplikasi-cek-bansos-2026-simak-syarat-dan-langkah-langkahnya</t>
+          <t>https://www.antaranews.com/berita/5670288/daftar-bansos-yang-masih-cair-tahun-ini-lengkap-dengan-syaratnya</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/IMG_8481.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/13/IMG-20260713-WA0009.jpg</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -841,33 +841,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>humaniora</t>
+          <t>hiburan</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Daftar bansos yang masih cair tahun ini, lengkap dengan syaratnya</t>
+          <t>Konser Kanye West di Jakarta 2026: Jadwal, harga tiket, dan cara beli resmi</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 07:11:38 +0700</t>
+          <t>Wed, 29 Jul 2026 07:53:10 +0700</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Pemerintah masih melanjutkan penyaluran sejumlah program bantuan sosial (bansos) sepanjang 2026 untuk membantu ...</t>
+          <t>Kabar yang dinantikan para penggemar akhirnya terwujud. Rapper asal Amerika Serikat, Kanye West atau yang kini dikenal ...</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5670288/daftar-bansos-yang-masih-cair-tahun-ini-lengkap-dengan-syaratnya</t>
+          <t>https://www.antaranews.com/berita/5670317/konser-kanye-west-di-jakarta-2026-jadwal-harga-tiket-dan-cara-beli-resmi</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/13/IMG-20260713-WA0009.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/04/26/1000102769.jpg</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -879,33 +879,33 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>hiburan</t>
+          <t>tekno</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15 Rekomendasi film bioskop seru bulan Agustus 2026</t>
+          <t>10 smartwatch terbaik 2026 untuk olahraga, lengkap dengan fitur dan rekomendasinya</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 16:37:40 +0700</t>
+          <t>Wed, 29 Jul 2026 07:40:37 +0700</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Memasuki Agustus 2026, deretan film baru siap meramaikan layar bioskop di Indonesia. Berbagai rumah produksi ...</t>
+          <t>Smartwatch olahraga semakin diminati karena menawarkan fitur pemantauan kesehatan, pelacakan aktivitas fisik, hingga ...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5671105/15-rekomendasi-film-bioskop-seru-bulan-agustus-2026</t>
+          <t>https://www.antaranews.com/berita/5670311/10-smartwatch-terbaik-2026-untuk-olahraga-lengkap-dengan-fitur-dan-rekomendasinya</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/03/20/1000292384.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/01/07/IMG-20240107-WA0013.jpg</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -917,33 +917,33 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>hiburan</t>
+          <t>tekno</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Konser Kanye West di Jakarta 2026: Jadwal, harga tiket, dan cara beli resmi</t>
+          <t>7 cara menjaga battery health iPhone agar tetap awet dan tak cepat turun</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 07:53:10 +0700</t>
+          <t>Wed, 29 Jul 2026 07:07:20 +0700</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Kabar yang dinantikan para penggemar akhirnya terwujud. Rapper asal Amerika Serikat, Kanye West atau yang kini dikenal ...</t>
+          <t>Kesehatan baterai atau Battery Health merupakan salah satu aspek penting yang perlu diperhatikan oleh pengguna iPhone. ...</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5670317/konser-kanye-west-di-jakarta-2026-jadwal-harga-tiket-dan-cara-beli-resmi</t>
+          <t>https://www.antaranews.com/berita/5670281/7-cara-menjaga-battery-health-iphone-agar-tetap-awet-dan-tak-cepat-turun</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2024/04/26/1000102769.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/29/InShot_20260629_204048450.jpg</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -955,33 +955,33 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>tekno</t>
+          <t>metro</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10 smartwatch terbaik 2026 untuk olahraga, lengkap dengan fitur dan rekomendasinya</t>
+          <t>Polisi buru bandar sabu pemasok dua pengedar di Jakarta Utara</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 07:40:37 +0700</t>
+          <t>Wed, 29 Jul 2026 20:47:46 +0700</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Smartwatch olahraga semakin diminati karena menawarkan fitur pemantauan kesehatan, pelacakan aktivitas fisik, hingga ...</t>
+          <t>Polsek Kawasan Sunda Kelapa, Jakarta Utara, masih memburu seorang bandar narkotika jenis sabu berinisial PN yang ...</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5670311/10-smartwatch-terbaik-2026-untuk-olahraga-lengkap-dengan-fitur-dan-rekomendasinya</t>
+          <t>https://www.antaranews.com/berita/5671636/polisi-buru-bandar-sabu-pemasok-dua-pengedar-di-jakarta-utara</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2024/01/07/IMG-20240107-WA0013.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/WhatsApp-Image-2026-07-29-at-20.16.31_1.jpeg</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -993,33 +993,33 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>tekno</t>
+          <t>hiburan</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7 cara menjaga battery health iPhone agar tetap awet dan tak cepat turun</t>
+          <t>15 Rekomendasi film bioskop seru bulan Agustus 2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 07:07:20 +0700</t>
+          <t>Wed, 29 Jul 2026 16:37:40 +0700</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Kesehatan baterai atau Battery Health merupakan salah satu aspek penting yang perlu diperhatikan oleh pengguna iPhone. ...</t>
+          <t>Memasuki Agustus 2026, deretan film baru siap meramaikan layar bioskop di Indonesia. Berbagai rumah produksi ...</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5670281/7-cara-menjaga-battery-health-iphone-agar-tetap-awet-dan-tak-cepat-turun</t>
+          <t>https://www.antaranews.com/berita/5671105/15-rekomendasi-film-bioskop-seru-bulan-agustus-2026</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/29/InShot_20260629_204048450.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/20/1000292384.jpg</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">

</xml_diff>